<commit_message>
Aplica as 4 correções do D2 decididas pelo autor
D2b-048: data de publicação da Res. CMN 5.274/2025 corrigida para o DOU de
22/12/2025 (também no normas-rag-corpus.md). D2b-050: retirada a descrição do
escopo dos decretos de 2025. D2-032: gabarito limitado ao texto do art. 1º da
Lei 15.263/2025. D2-036: gabarito com os três incisos do art. 2º, § 1º, da
Res. CMN 4.893/2021. Vigência de cada dispositivo conferida antes de aplicar
(registro em CONFERENCIA-TEXTOS.md).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/d2-rag/revisao-autor.xlsx
+++ b/dados/d2-rag/revisao-autor.xlsx
@@ -493,7 +493,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Gerada por dados/d2-rag/gerar-revisao.py a partir de d2-perguntas.csv (SHA-256 92b04cb68311f48875ef4d4dc6eae61f082b18e0c80bb510523ca6d14dc1b822).</t>
+          <t>Gerada por dados/d2-rag/gerar-revisao.py a partir de d2-perguntas.csv (SHA-256 81d2c66871729bec1cf3db1a8c9c87d7271091164bcc0c980b0c269a6c2dc222).</t>
         </is>
       </c>
     </row>
@@ -2566,7 +2566,7 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Lei no 15.263/2025</t>
+          <t>art. 1o</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
@@ -2576,7 +2576,7 @@
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>Instituiu a Politica Nacional de Linguagem Simples, vinculante para toda a administracao publica, o que alcanca os bancos publicos.</t>
+          <t>Instituiu a Politica Nacional de Linguagem Simples, a ser observada pelos orgaos e entidades da administracao publica direta e indireta de todos os Poderes da Uniao, dos Estados, do Distrito Federal e dos Municipios, em sua comunicacao com a populacao (art. 1o).</t>
         </is>
       </c>
       <c r="I33" s="4" t="inlineStr">
@@ -2599,10 +2599,18 @@
           <t>Manter, mas deixar a interpretação explícita, ou limitar o gabarito ao texto do art. 1º</t>
         </is>
       </c>
-      <c r="M33" s="6" t="inlineStr"/>
+      <c r="M33" s="6" t="inlineStr">
+        <is>
+          <t>Manter com ajuste</t>
+        </is>
+      </c>
       <c r="N33" s="6" t="inlineStr"/>
       <c r="O33" s="6" t="inlineStr"/>
-      <c r="P33" s="6" t="inlineStr"/>
+      <c r="P33" s="6" t="inlineStr">
+        <is>
+          <t>Decidido em 02/10/2026 e aplicado no d2-perguntas.csv: Opção b (só o texto da lei). Texto do art. 1º, sem a inferência sobre bancos públicos; `dispositivo` passa a "art. 1o"</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -2828,7 +2836,7 @@
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>Nao. Deve ser compativel com o porte, o perfil de risco e o modelo de negocio da instituicao.</t>
+          <t>Nao. Deve ser compativel com (I) o porte, o perfil de risco e o modelo de negocio da instituicao; (II) a natureza das operacoes e a complexidade dos produtos, servicos, atividades e processos da instituicao; e (III) a sensibilidade dos dados e das informacoes sob responsabilidade da instituicao.</t>
         </is>
       </c>
       <c r="I37" s="4" t="inlineStr">
@@ -2851,10 +2859,18 @@
           <t>Completar com os incisos II e III, ou aceitar o inciso I como resposta suficiente</t>
         </is>
       </c>
-      <c r="M37" s="6" t="inlineStr"/>
+      <c r="M37" s="6" t="inlineStr">
+        <is>
+          <t>Manter com ajuste</t>
+        </is>
+      </c>
       <c r="N37" s="6" t="inlineStr"/>
       <c r="O37" s="6" t="inlineStr"/>
-      <c r="P37" s="6" t="inlineStr"/>
+      <c r="P37" s="6" t="inlineStr">
+        <is>
+          <t>Decidido em 02/10/2026 e aplicado no d2-perguntas.csv: Completar. Os três incisos do art. 2º, § 1º</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -3556,7 +3572,7 @@
       </c>
       <c r="H49" s="4" t="inlineStr">
         <is>
-          <t>Ate 1o de marco de 2026. A norma foi publicada em 18/12/2025 e entrou em vigor na data da publicacao.</t>
+          <t>Ate 1o de marco de 2026. A resolucao, de 18/12/2025, foi publicada no DOU de 22/12/2025 e entrou em vigor na data da publicacao.</t>
         </is>
       </c>
       <c r="I49" s="4" t="inlineStr">
@@ -3579,10 +3595,18 @@
           <t>"Até 1º de março de 2026. A resolução, de 18/12/2025, foi publicada no DOU de 22/12/2025 e entrou em vigor na data da publicação." O mesmo erro está em `bibliografia/normas-rag-corpus.md`, item 6</t>
         </is>
       </c>
-      <c r="M49" s="6" t="inlineStr"/>
+      <c r="M49" s="6" t="inlineStr">
+        <is>
+          <t>Manter com ajuste</t>
+        </is>
+      </c>
       <c r="N49" s="6" t="inlineStr"/>
       <c r="O49" s="6" t="inlineStr"/>
-      <c r="P49" s="6" t="inlineStr"/>
+      <c r="P49" s="6" t="inlineStr">
+        <is>
+          <t>Decidido em 02/10/2026 e aplicado no d2-perguntas.csv: Corrigir. Resolução de 18/12/2025, publicada no DOU de 22/12/2025, em vigor na publicação; prazo até 1º/03/2026. Corrigido também em `bibliografia/normas-rag-corpus.md`, item 6</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
@@ -3684,7 +3708,7 @@
       </c>
       <c r="H51" s="4" t="inlineStr">
         <is>
-          <t>Nao. O art. 32 e o Anexo do Decreto no 6.306/2007 nao foram alterados pelos Decretos no 12.466, 12.467 e 12.499, de 2025, que trataram de IOF sobre credito, cambio e seguro.</t>
+          <t>Nao. O art. 32 e o Anexo do Decreto no 6.306/2007 nao foram alterados pelos Decretos no 12.466, 12.467 e 12.499, de 2025.</t>
         </is>
       </c>
       <c r="I51" s="4" t="inlineStr">
@@ -3707,10 +3731,18 @@
           <t>Trocar "que trataram de IOF sobre crédito, câmbio e seguro" por uma redação que não afirme o escopo completo dos decretos, ou mencione o art. 32-D</t>
         </is>
       </c>
-      <c r="M51" s="6" t="inlineStr"/>
+      <c r="M51" s="6" t="inlineStr">
+        <is>
+          <t>Manter com ajuste</t>
+        </is>
+      </c>
       <c r="N51" s="6" t="inlineStr"/>
       <c r="O51" s="6" t="inlineStr"/>
-      <c r="P51" s="6" t="inlineStr"/>
+      <c r="P51" s="6" t="inlineStr">
+        <is>
+          <t>Decidido em 02/10/2026 e aplicado no d2-perguntas.csv: Corrigir. Retirado o trecho que descrevia o escopo dos decretos de 2025</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Ajusta a metodologia ao tamanho real do D2 e tira a ANBIMA do conjunto de teste
Decisão do autor (02/10/2026): nenhum item excluído; o texto passa de "30 a 50
perguntas" para 39 perguntas mais um subconjunto adicional de 12 sobre vigência,
e descreve as fontes que o D2 de fato cobre (CVM, CMN e legislação federal de
tributação e de linguagem simples).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/d2-rag/revisao-autor.xlsx
+++ b/dados/d2-rag/revisao-autor.xlsx
@@ -3883,7 +3883,11 @@
           <t>a) excluir um item (a revisão da aba Itens pode indicar qual); b) ajustar a redação do texto da dissertação para 51.</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr"/>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>b) 02/10/2026: nenhum item excluído; metodologia ajustada para 39 perguntas mais subconjunto adicional de 12 de vigência, sem citar a ANBIMA (sem item no D2).</t>
+        </is>
+      </c>
       <c r="F2" s="6" t="inlineStr"/>
     </row>
     <row r="3">
@@ -3931,7 +3935,11 @@
           <t>Decidir item a item na aba Itens (coluna decisao_autor).</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr"/>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>02/10/2026: as 4 correções aplicadas (ver aba Itens e CONFERENCIA-TEXTOS.md).</t>
+        </is>
+      </c>
       <c r="F4" s="6" t="inlineStr"/>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Fixa as métricas da validação da base RAG
Decisão do autor (02/10/2026): recall@k com k = 1, 3, 5 e 10 e MRR no lugar da
precisão (com um dispositivo correto por pergunta, a precisão@k fica limitada a
1/k); no D2b, proporção de perguntas com a redação vigente recuperada antes da
revogada. k operacional provisório 5, a confirmar pela curva de recall.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/d2-rag/revisao-autor.xlsx
+++ b/dados/d2-rag/revisao-autor.xlsx
@@ -3911,7 +3911,11 @@
           <t>Um k único ou uma série de valores reportados lado a lado (decisão do autor).</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr"/>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>c) 02/10/2026: recall@k com k = 1, 3, 5 e 10 e MRR no lugar da precisão; no D2b, proporção com a redação vigente antes da revogada; k operacional provisório 5, a confirmar pela curva de recall.</t>
+        </is>
+      </c>
       <c r="F3" s="6" t="inlineStr"/>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
D2: conferência dos 28 itens restantes contra o texto vigente
Corrige D2-038 (a Res. CMN 4.557 se aplica de S1 a S4; o S5 foi revogado
pela 5.049/2022) e D2b-051 (a versão 13 incorpora as 5.222 e 5.226/2025; a
5.207/2025 produz efeitos em 01/01/2027), por decisão do autor. Atualiza a
nota da 4.557 no corpus (versão 13, link _L) e registra a vigência da CVM 30
e o risco de revisão na agenda regulatória de 2026.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/d2-rag/revisao-autor.xlsx
+++ b/dados/d2-rag/revisao-autor.xlsx
@@ -37,7 +37,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -46,17 +46,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EFEFEF"/>
+        <fgColor rgb="00D9EAD3"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DDEBF7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9EAD3"/>
       </patternFill>
     </fill>
     <fill>
@@ -82,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -104,9 +99,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -474,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -493,7 +485,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Gerada por dados/d2-rag/gerar-revisao.py a partir de d2-perguntas.csv (SHA-256 81d2c66871729bec1cf3db1a8c9c87d7271091164bcc0c980b0c269a6c2dc222).</t>
+          <t>Gerada por dados/d2-rag/gerar-revisao.py a partir de d2-perguntas.csv (SHA-256 152cc8485237de9dfe866e439d36fd2f3b353d467972b6d58ab7288a95f27f26).</t>
         </is>
       </c>
     </row>
@@ -548,43 +540,29 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Erro de fato / Ressalva / Confere — resultado da conferência de 02/10/2026 contra o texto legível</t>
+          <t xml:space="preserve">  Erro de fato / Ressalva / Confere — resultado da conferência contra o texto vigente</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (ver CONFERENCIA-TEXTOS.md);</t>
+          <t xml:space="preserve">  (ver CONFERENCIA-TEXTOS.md): 23 itens em 02/10/2026 e os 28 restantes (Res. CVM 30/2021 e</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Fora da conferência — itens cuja fonte é PDF com camada de texto (Res. CVM 30/2021 e Res. CMN</t>
+          <t xml:space="preserve">  Res. CMN 4.557/2017) em 03/10/2026. Os 51 itens estão conferidos.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  4.557/2017), que não entraram naquela conferência. A revisão do autor é a primeira leitura deles</t>
-        </is>
-      </c>
+      <c r="A15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  depois da geração.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
         <is>
           <t>Aba Decisoes: questões de desenho do D2 que são do autor. A coluna escolha_autor fica em branco.</t>
         </is>
@@ -752,10 +730,14 @@
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>Fora da conferência</t>
-        </is>
-      </c>
-      <c r="K2" s="4" t="inlineStr"/>
+          <t>Confere</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
+          <t>CVM 30, art. 2º — consolidado CVM: Integrantes do sistema de distribuição e consultores não podem recomendar sem verificar a adequação ao perfil</t>
+        </is>
+      </c>
       <c r="L2" s="4" t="inlineStr"/>
       <c r="M2" s="6" t="inlineStr"/>
       <c r="N2" s="6" t="inlineStr"/>
@@ -810,10 +792,14 @@
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>Fora da conferência</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr"/>
+          <t>Confere</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>CVM 30, art. 3º, caput — consolidado CVM: Incisos I a III: objetivos, situação financeira e conhecimento do cliente</t>
+        </is>
+      </c>
       <c r="L3" s="4" t="inlineStr"/>
       <c r="M3" s="6" t="inlineStr"/>
       <c r="N3" s="6" t="inlineStr"/>
@@ -868,10 +854,14 @@
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>Fora da conferência</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr"/>
+          <t>Confere</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>CVM 30, art. 3º, § 1º — consolidado CVM: Período do investimento, preferências quanto à assunção de riscos e finalidades</t>
+        </is>
+      </c>
       <c r="L4" s="4" t="inlineStr"/>
       <c r="M4" s="6" t="inlineStr"/>
       <c r="N4" s="6" t="inlineStr"/>
@@ -926,10 +916,14 @@
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>Fora da conferência</t>
-        </is>
-      </c>
-      <c r="K5" s="4" t="inlineStr"/>
+          <t>Confere</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>CVM 30, art. 3º, § 2º — consolidado CVM: Receitas regulares, patrimônio e necessidade futura de recursos</t>
+        </is>
+      </c>
       <c r="L5" s="4" t="inlineStr"/>
       <c r="M5" s="6" t="inlineStr"/>
       <c r="N5" s="6" t="inlineStr"/>
@@ -984,10 +978,14 @@
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>Fora da conferência</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="inlineStr"/>
+          <t>Confere</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>CVM 30, art. 3º, § 3º — consolidado CVM: Familiaridade; natureza, volume, frequência e período das operações; formação e experiência</t>
+        </is>
+      </c>
       <c r="L6" s="4" t="inlineStr"/>
       <c r="M6" s="6" t="inlineStr"/>
       <c r="N6" s="6" t="inlineStr"/>
@@ -1042,10 +1040,14 @@
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>Fora da conferência</t>
-        </is>
-      </c>
-      <c r="K7" s="4" t="inlineStr"/>
+          <t>Confere</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>CVM 30, art. 3º, § 4º — consolidado CVM: O inciso III do § 3º não se aplica a cliente pessoa jurídica</t>
+        </is>
+      </c>
       <c r="L7" s="4" t="inlineStr"/>
       <c r="M7" s="6" t="inlineStr"/>
       <c r="N7" s="6" t="inlineStr"/>
@@ -1100,10 +1102,14 @@
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>Fora da conferência</t>
-        </is>
-      </c>
-      <c r="K8" s="4" t="inlineStr"/>
+          <t>Confere</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>CVM 30, art. 3º, § 5º — consolidado CVM: Custos diretos e indiretos; abster-se de recomendar custos excessivos e inadequados ao perfil</t>
+        </is>
+      </c>
       <c r="L8" s="4" t="inlineStr"/>
       <c r="M8" s="6" t="inlineStr"/>
       <c r="N8" s="6" t="inlineStr"/>
@@ -1158,10 +1164,14 @@
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>Fora da conferência</t>
-        </is>
-      </c>
-      <c r="K9" s="4" t="inlineStr"/>
+          <t>Confere</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>CVM 30, art. 4º — consolidado CVM: Classificar o cliente em categorias de perfil de risco previamente estabelecidas</t>
+        </is>
+      </c>
       <c r="L9" s="4" t="inlineStr"/>
       <c r="M9" s="6" t="inlineStr"/>
       <c r="N9" s="6" t="inlineStr"/>
@@ -1216,10 +1226,14 @@
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>Fora da conferência</t>
-        </is>
-      </c>
-      <c r="K10" s="4" t="inlineStr"/>
+          <t>Confere</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>CVM 30, art. 5º, par. único — consolidado CVM: Riscos, perfil dos emissores e prestadores, garantias e prazos de carência</t>
+        </is>
+      </c>
       <c r="L10" s="4" t="inlineStr"/>
       <c r="M10" s="6" t="inlineStr"/>
       <c r="N10" s="6" t="inlineStr"/>
@@ -1274,10 +1288,14 @@
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>Fora da conferência</t>
-        </is>
-      </c>
-      <c r="K11" s="4" t="inlineStr"/>
+          <t>Confere</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>CVM 30, art. 6º — consolidado CVM: Vedação nas hipóteses dos incisos I a III</t>
+        </is>
+      </c>
       <c r="L11" s="4" t="inlineStr"/>
       <c r="M11" s="6" t="inlineStr"/>
       <c r="N11" s="6" t="inlineStr"/>
@@ -1332,10 +1350,14 @@
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>Fora da conferência</t>
-        </is>
-      </c>
-      <c r="K12" s="4" t="inlineStr"/>
+          <t>Confere</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>CVM 30, art. 7º — consolidado CVM: Alerta com as causas da divergência e declaração expressa, antes da primeira operação com a categoria</t>
+        </is>
+      </c>
       <c r="L12" s="4" t="inlineStr"/>
       <c r="M12" s="6" t="inlineStr"/>
       <c r="N12" s="6" t="inlineStr"/>
@@ -1390,10 +1412,14 @@
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>Fora da conferência</t>
-        </is>
-      </c>
-      <c r="K13" s="4" t="inlineStr"/>
+          <t>Confere</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>CVM 30, art. 7º, par. único — consolidado CVM: Dispensa quando o cliente implementa recomendações de consultor autorizado pela CVM</t>
+        </is>
+      </c>
       <c r="L13" s="4" t="inlineStr"/>
       <c r="M13" s="6" t="inlineStr"/>
       <c r="N13" s="6" t="inlineStr"/>
@@ -1448,10 +1474,14 @@
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>Fora da conferência</t>
-        </is>
-      </c>
-      <c r="K14" s="4" t="inlineStr"/>
+          <t>Confere</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>CVM 30, art. 8º, § 1º — consolidado CVM: Nomeação ou substituição do diretor informada à CVM em 7 dias úteis</t>
+        </is>
+      </c>
       <c r="L14" s="4" t="inlineStr"/>
       <c r="M14" s="6" t="inlineStr"/>
       <c r="N14" s="6" t="inlineStr"/>
@@ -1506,10 +1536,14 @@
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>Fora da conferência</t>
-        </is>
-      </c>
-      <c r="K15" s="4" t="inlineStr"/>
+          <t>Confere</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>CVM 30, art. 8º, § 2º — consolidado CVM: Relatório até o último dia útil de abril, relativo ao ano civil anterior</t>
+        </is>
+      </c>
       <c r="L15" s="4" t="inlineStr"/>
       <c r="M15" s="6" t="inlineStr"/>
       <c r="N15" s="6" t="inlineStr"/>
@@ -1564,10 +1598,14 @@
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>Fora da conferência</t>
-        </is>
-      </c>
-      <c r="K16" s="4" t="inlineStr"/>
+          <t>Confere</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>CVM 30, art. 9º, I — consolidado CVM: Critérios da norma de PLDFT, com intervalo máximo de 5 anos</t>
+        </is>
+      </c>
       <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="6" t="inlineStr"/>
       <c r="N16" s="6" t="inlineStr"/>
@@ -1622,10 +1660,14 @@
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>Fora da conferência</t>
-        </is>
-      </c>
-      <c r="K17" s="4" t="inlineStr"/>
+          <t>Confere</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>CVM 30, art. 9º, II — consolidado CVM: Nova classificação dos produtos em intervalos não superiores a 24 meses</t>
+        </is>
+      </c>
       <c r="L17" s="4" t="inlineStr"/>
       <c r="M17" s="6" t="inlineStr"/>
       <c r="N17" s="6" t="inlineStr"/>
@@ -1680,10 +1722,14 @@
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>Fora da conferência</t>
-        </is>
-      </c>
-      <c r="K18" s="4" t="inlineStr"/>
+          <t>Confere</t>
+        </is>
+      </c>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t>CVM 30, art. 10 — consolidado CVM: Incisos I a IV; o inciso I exceciona as pessoas naturais do art. 11, IV e do art. 12, II e III</t>
+        </is>
+      </c>
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="6" t="inlineStr"/>
       <c r="N18" s="6" t="inlineStr"/>
@@ -1738,10 +1784,14 @@
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>Fora da conferência</t>
-        </is>
-      </c>
-      <c r="K19" s="4" t="inlineStr"/>
+          <t>Confere</t>
+        </is>
+      </c>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>CVM 30, art. 11, IV — consolidado CVM: Aplicações superiores a R$ 10.000.000,00, com atestado por escrito (Anexo A)</t>
+        </is>
+      </c>
       <c r="L19" s="4" t="inlineStr"/>
       <c r="M19" s="6" t="inlineStr"/>
       <c r="N19" s="6" t="inlineStr"/>
@@ -1796,10 +1846,14 @@
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>Fora da conferência</t>
-        </is>
-      </c>
-      <c r="K20" s="4" t="inlineStr"/>
+          <t>Confere</t>
+        </is>
+      </c>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t>CVM 30, art. 12, II — consolidado CVM: Aplicações superiores a R$ 1.000.000,00, com atestado por escrito (Anexo B)</t>
+        </is>
+      </c>
       <c r="L20" s="4" t="inlineStr"/>
       <c r="M20" s="6" t="inlineStr"/>
       <c r="N20" s="6" t="inlineStr"/>
@@ -1854,10 +1908,14 @@
       </c>
       <c r="J21" s="5" t="inlineStr">
         <is>
-          <t>Fora da conferência</t>
-        </is>
-      </c>
-      <c r="K21" s="4" t="inlineStr"/>
+          <t>Confere</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>CVM 30, art. 14 — consolidado CVM: Mínimo de 5 anos da última recomendação ou operação, ou prazo superior determinado pela CVM</t>
+        </is>
+      </c>
       <c r="L21" s="4" t="inlineStr"/>
       <c r="M21" s="6" t="inlineStr"/>
       <c r="N21" s="6" t="inlineStr"/>
@@ -1912,10 +1970,14 @@
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>Fora da conferência</t>
-        </is>
-      </c>
-      <c r="K22" s="4" t="inlineStr"/>
+          <t>Confere</t>
+        </is>
+      </c>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>CVM 30, art. 16 — consolidado CVM: Infração grave (art. 11, § 3º, da Lei nº 6.385/1976) a inobservância dos arts. 6º e 7º</t>
+        </is>
+      </c>
       <c r="L22" s="4" t="inlineStr"/>
       <c r="M22" s="6" t="inlineStr"/>
       <c r="N22" s="6" t="inlineStr"/>
@@ -1970,10 +2032,14 @@
       </c>
       <c r="J23" s="5" t="inlineStr">
         <is>
-          <t>Fora da conferência</t>
-        </is>
-      </c>
-      <c r="K23" s="4" t="inlineStr"/>
+          <t>Confere</t>
+        </is>
+      </c>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>CVM 30, art. 18 — consolidado CVM: Em vigor em 1º/06/2021</t>
+        </is>
+      </c>
       <c r="L23" s="4" t="inlineStr"/>
       <c r="M23" s="6" t="inlineStr"/>
       <c r="N23" s="6" t="inlineStr"/>
@@ -2026,7 +2092,7 @@
           <t>bibliografia/normas/resolucao-cmn-4222-2013-regulamento-fgc.pdf</t>
         </is>
       </c>
-      <c r="J24" s="7" t="inlineStr">
+      <c r="J24" s="5" t="inlineStr">
         <is>
           <t>Confere</t>
         </is>
@@ -2088,7 +2154,7 @@
           <t>bibliografia/normas/resolucao-cmn-4222-2013-regulamento-fgc.pdf</t>
         </is>
       </c>
-      <c r="J25" s="7" t="inlineStr">
+      <c r="J25" s="5" t="inlineStr">
         <is>
           <t>Confere</t>
         </is>
@@ -2150,7 +2216,7 @@
           <t>bibliografia/normas/resolucao-cmn-4222-2013-regulamento-fgc.pdf</t>
         </is>
       </c>
-      <c r="J26" s="7" t="inlineStr">
+      <c r="J26" s="5" t="inlineStr">
         <is>
           <t>Confere</t>
         </is>
@@ -2212,7 +2278,7 @@
           <t>bibliografia/normas/resolucao-cmn-4222-2013-regulamento-fgc.pdf</t>
         </is>
       </c>
-      <c r="J27" s="7" t="inlineStr">
+      <c r="J27" s="5" t="inlineStr">
         <is>
           <t>Confere</t>
         </is>
@@ -2274,7 +2340,7 @@
           <t>bibliografia/normas/lei-11033-2004-ir-compilado.pdf</t>
         </is>
       </c>
-      <c r="J28" s="7" t="inlineStr">
+      <c r="J28" s="5" t="inlineStr">
         <is>
           <t>Confere</t>
         </is>
@@ -2336,7 +2402,7 @@
           <t>bibliografia/normas/lei-11033-2004-ir-compilado.pdf</t>
         </is>
       </c>
-      <c r="J29" s="7" t="inlineStr">
+      <c r="J29" s="5" t="inlineStr">
         <is>
           <t>Confere</t>
         </is>
@@ -2398,7 +2464,7 @@
           <t>bibliografia/normas/decreto-6306-2007-iof-compilado.pdf</t>
         </is>
       </c>
-      <c r="J30" s="7" t="inlineStr">
+      <c r="J30" s="5" t="inlineStr">
         <is>
           <t>Confere</t>
         </is>
@@ -2460,7 +2526,7 @@
           <t>bibliografia/normas/decreto-6306-2007-iof-compilado.pdf</t>
         </is>
       </c>
-      <c r="J31" s="7" t="inlineStr">
+      <c r="J31" s="5" t="inlineStr">
         <is>
           <t>Confere</t>
         </is>
@@ -2522,7 +2588,7 @@
           <t>bibliografia/normas/decreto-6306-2007-iof-compilado.pdf</t>
         </is>
       </c>
-      <c r="J32" s="7" t="inlineStr">
+      <c r="J32" s="5" t="inlineStr">
         <is>
           <t>Confere</t>
         </is>
@@ -2584,7 +2650,7 @@
           <t>bibliografia/normas/lei-15263-2025-linguagem-simples.pdf</t>
         </is>
       </c>
-      <c r="J33" s="8" t="inlineStr">
+      <c r="J33" s="7" t="inlineStr">
         <is>
           <t>Ressalva</t>
         </is>
@@ -2658,7 +2724,7 @@
           <t>bibliografia/normas/lei-15263-2025-linguagem-simples.pdf</t>
         </is>
       </c>
-      <c r="J34" s="7" t="inlineStr">
+      <c r="J34" s="5" t="inlineStr">
         <is>
           <t>Confere</t>
         </is>
@@ -2720,7 +2786,7 @@
           <t>bibliografia/normas/resolucao-cmn-4968-2021-controles-internos.pdf</t>
         </is>
       </c>
-      <c r="J35" s="7" t="inlineStr">
+      <c r="J35" s="5" t="inlineStr">
         <is>
           <t>Confere</t>
         </is>
@@ -2782,7 +2848,7 @@
           <t>bibliografia/normas/resolucao-cmn-4879-2020-auditoria-interna.pdf</t>
         </is>
       </c>
-      <c r="J36" s="7" t="inlineStr">
+      <c r="J36" s="5" t="inlineStr">
         <is>
           <t>Confere</t>
         </is>
@@ -2844,7 +2910,7 @@
           <t>bibliografia/normas/resolucao-cmn-4893-2021-seguranca-cibernetica.pdf</t>
         </is>
       </c>
-      <c r="J37" s="8" t="inlineStr">
+      <c r="J37" s="7" t="inlineStr">
         <is>
           <t>Ressalva</t>
         </is>
@@ -2918,7 +2984,7 @@
           <t>bibliografia/normas/resolucao-cmn-4893-2021-seguranca-cibernetica.pdf</t>
         </is>
       </c>
-      <c r="J38" s="7" t="inlineStr">
+      <c r="J38" s="5" t="inlineStr">
         <is>
           <t>Confere</t>
         </is>
@@ -2962,7 +3028,7 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>estrutura geral</t>
+          <t>art. 2o, § 1o</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
@@ -2972,7 +3038,7 @@
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>Sim. A norma organiza as exigencias por segmento prudencial (S1 a S5) e exige a Declaracao de Apetite por Riscos (RAS) e programa de testes de estresse.</t>
+          <t>Sim. As estruturas de gerenciamento devem ser compativeis com o modelo de negocio, a natureza das operacoes e a complexidade dos produtos, servicos, atividades e processos da instituicao; proporcionais a dimensao e a relevancia da exposicao aos riscos; e adequadas ao perfil de riscos e a importancia sistemica da instituicao. A resolucao se aplica as instituicoes dos segmentos S1 a S4.</t>
         </is>
       </c>
       <c r="I39" s="4" t="inlineStr">
@@ -2980,17 +3046,33 @@
           <t>bibliografia/normas/resolucao-cmn-4557-2017-gerenciamento-riscos-capital.pdf</t>
         </is>
       </c>
-      <c r="J39" s="5" t="inlineStr">
-        <is>
-          <t>Fora da conferência</t>
-        </is>
-      </c>
-      <c r="K39" s="4" t="inlineStr"/>
-      <c r="L39" s="4" t="inlineStr"/>
-      <c r="M39" s="6" t="inlineStr"/>
+      <c r="J39" s="8" t="inlineStr">
+        <is>
+          <t>Erro de fato</t>
+        </is>
+      </c>
+      <c r="K39" s="4" t="inlineStr">
+        <is>
+          <t>O art. 2º aplica a resolução aos segmentos S1 a S4; o capítulo do S5 (arts. 61 a 64) foi revogado pela Res. CMN nº 5.049/2022 a partir de 1º/01/2023. O gabarito dizia "S1 a S5", e o dispositivo era "estrutura geral"</t>
+        </is>
+      </c>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t>Dispositivo "art. 2º, § 1º"; gabarito com os critérios do § 1º (compatibilidade, proporcionalidade e adequação ao perfil de riscos) e o escopo S1 a S4</t>
+        </is>
+      </c>
+      <c r="M39" s="6" t="inlineStr">
+        <is>
+          <t>Manter com ajuste</t>
+        </is>
+      </c>
       <c r="N39" s="6" t="inlineStr"/>
       <c r="O39" s="6" t="inlineStr"/>
-      <c r="P39" s="6" t="inlineStr"/>
+      <c r="P39" s="6" t="inlineStr">
+        <is>
+          <t>Decidido em 03/10/2026 e aplicado no d2-perguntas.csv: Corrigir. Critérios do art. 2º, § 1º e escopo S1 a S4; dispositivo "art. 2º, § 1º"</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -3038,7 +3120,7 @@
           <t>bibliografia/normas/resolucao-cmn-5274-2025-altera-4893.pdf</t>
         </is>
       </c>
-      <c r="J40" s="7" t="inlineStr">
+      <c r="J40" s="5" t="inlineStr">
         <is>
           <t>Confere</t>
         </is>
@@ -3102,10 +3184,14 @@
       </c>
       <c r="J41" s="5" t="inlineStr">
         <is>
-          <t>Fora da conferência</t>
-        </is>
-      </c>
-      <c r="K41" s="4" t="inlineStr"/>
+          <t>Confere</t>
+        </is>
+      </c>
+      <c r="K41" s="4" t="inlineStr">
+        <is>
+          <t>CVM 30, art. 11, VII — consolidado CVM: Três redações empilhadas; a vigente, da Res. CVM nº 179/2023, diz "assessores de investimento"</t>
+        </is>
+      </c>
       <c r="L41" s="4" t="inlineStr"/>
       <c r="M41" s="6" t="inlineStr"/>
       <c r="N41" s="6" t="inlineStr"/>
@@ -3160,10 +3246,14 @@
       </c>
       <c r="J42" s="5" t="inlineStr">
         <is>
-          <t>Fora da conferência</t>
-        </is>
-      </c>
-      <c r="K42" s="4" t="inlineStr"/>
+          <t>Confere</t>
+        </is>
+      </c>
+      <c r="K42" s="4" t="inlineStr">
+        <is>
+          <t>CVM 30, art. 12, III — consolidado CVM: Redação da Res. CVM nº 179/2023: "assessores de investimento"</t>
+        </is>
+      </c>
       <c r="L42" s="4" t="inlineStr"/>
       <c r="M42" s="6" t="inlineStr"/>
       <c r="N42" s="6" t="inlineStr"/>
@@ -3218,10 +3308,14 @@
       </c>
       <c r="J43" s="5" t="inlineStr">
         <is>
-          <t>Fora da conferência</t>
-        </is>
-      </c>
-      <c r="K43" s="4" t="inlineStr"/>
+          <t>Confere</t>
+        </is>
+      </c>
+      <c r="K43" s="4" t="inlineStr">
+        <is>
+          <t>CVM 30, art. 11, IX — consolidado CVM: Fundos patrimoniais, inciso incluído pela Res. CVM nº 162/2022</t>
+        </is>
+      </c>
       <c r="L43" s="4" t="inlineStr"/>
       <c r="M43" s="6" t="inlineStr"/>
       <c r="N43" s="6" t="inlineStr"/>
@@ -3276,10 +3370,14 @@
       </c>
       <c r="J44" s="5" t="inlineStr">
         <is>
-          <t>Fora da conferência</t>
-        </is>
-      </c>
-      <c r="K44" s="4" t="inlineStr"/>
+          <t>Confere</t>
+        </is>
+      </c>
+      <c r="K44" s="4" t="inlineStr">
+        <is>
+          <t>CVM 30, art. 17 — consolidado CVM: Revoga a Instrução CVM nº 539/2013</t>
+        </is>
+      </c>
       <c r="L44" s="4" t="inlineStr"/>
       <c r="M44" s="6" t="inlineStr"/>
       <c r="N44" s="6" t="inlineStr"/>
@@ -3332,7 +3430,7 @@
           <t>bibliografia/normas/resolucao-cmn-4893-2021-seguranca-cibernetica.pdf</t>
         </is>
       </c>
-      <c r="J45" s="7" t="inlineStr">
+      <c r="J45" s="5" t="inlineStr">
         <is>
           <t>Confere</t>
         </is>
@@ -3394,7 +3492,7 @@
           <t>bibliografia/normas/resolucao-cmn-4893-2021-seguranca-cibernetica.pdf</t>
         </is>
       </c>
-      <c r="J46" s="7" t="inlineStr">
+      <c r="J46" s="5" t="inlineStr">
         <is>
           <t>Confere</t>
         </is>
@@ -3456,7 +3554,7 @@
           <t>bibliografia/normas/resolucao-cmn-4879-2020-auditoria-interna.pdf</t>
         </is>
       </c>
-      <c r="J47" s="7" t="inlineStr">
+      <c r="J47" s="5" t="inlineStr">
         <is>
           <t>Confere</t>
         </is>
@@ -3518,7 +3616,7 @@
           <t>bibliografia/normas/resolucao-cmn-4968-2021-controles-internos.pdf</t>
         </is>
       </c>
-      <c r="J48" s="7" t="inlineStr">
+      <c r="J48" s="5" t="inlineStr">
         <is>
           <t>Confere</t>
         </is>
@@ -3580,7 +3678,7 @@
           <t>bibliografia/normas/resolucao-cmn-5274-2025-altera-4893.pdf</t>
         </is>
       </c>
-      <c r="J49" s="9" t="inlineStr">
+      <c r="J49" s="8" t="inlineStr">
         <is>
           <t>Erro de fato</t>
         </is>
@@ -3654,7 +3752,7 @@
           <t>bibliografia/normas/lei-11033-2004-ir-compilado.pdf</t>
         </is>
       </c>
-      <c r="J50" s="7" t="inlineStr">
+      <c r="J50" s="5" t="inlineStr">
         <is>
           <t>Confere</t>
         </is>
@@ -3716,7 +3814,7 @@
           <t>bibliografia/normas/decreto-6306-2007-iof-compilado.pdf</t>
         </is>
       </c>
-      <c r="J51" s="8" t="inlineStr">
+      <c r="J51" s="7" t="inlineStr">
         <is>
           <t>Ressalva</t>
         </is>
@@ -3782,7 +3880,7 @@
       </c>
       <c r="H52" s="4" t="inlineStr">
         <is>
-          <t>Nao. A ementa tem redacao dada pela Resolucao no 4.745/2019, e o texto consolidado incorpora alteracoes ate a Resolucao CMN no 5.194/2024.</t>
+          <t>Nao. A ementa tem redacao dada pela Resolucao no 4.745/2019. Entre as alteracoes de 2025, as Resolucoes CMN no 5.222 e 5.226 ja estao em vigor, e a no 5.207 produz efeitos a partir de 1o/01/2027.</t>
         </is>
       </c>
       <c r="I52" s="4" t="inlineStr">
@@ -3790,17 +3888,33 @@
           <t>bibliografia/normas/resolucao-cmn-4557-2017-gerenciamento-riscos-capital.pdf</t>
         </is>
       </c>
-      <c r="J52" s="5" t="inlineStr">
-        <is>
-          <t>Fora da conferência</t>
-        </is>
-      </c>
-      <c r="K52" s="4" t="inlineStr"/>
-      <c r="L52" s="4" t="inlineStr"/>
-      <c r="M52" s="6" t="inlineStr"/>
+      <c r="J52" s="8" t="inlineStr">
+        <is>
+          <t>Erro de fato</t>
+        </is>
+      </c>
+      <c r="K52" s="4" t="inlineStr">
+        <is>
+          <t>A versão 13 incorpora as Res. CMN nº 5.222/2025 e 5.226/2025, não "alterações até a 5.194/2024"; a Res. CMN nº 5.207/2025 altera o art. 25 a partir de 1º/01/2027</t>
+        </is>
+      </c>
+      <c r="L52" s="4" t="inlineStr">
+        <is>
+          <t>Ementa com redação da 4.745/2019; 5.222 e 5.226 em vigor; 5.207 com efeitos a partir de 1º/01/2027</t>
+        </is>
+      </c>
+      <c r="M52" s="6" t="inlineStr">
+        <is>
+          <t>Manter com ajuste</t>
+        </is>
+      </c>
       <c r="N52" s="6" t="inlineStr"/>
       <c r="O52" s="6" t="inlineStr"/>
-      <c r="P52" s="6" t="inlineStr"/>
+      <c r="P52" s="6" t="inlineStr">
+        <is>
+          <t>Decidido em 03/10/2026 e aplicado no d2-perguntas.csv: Corrigir. Ementa da 4.745/2019; 5.222 e 5.226 em vigor; 5.207 a partir de 1º/01/2027</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:P52"/>
@@ -3941,7 +4055,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>02/10/2026: as 4 correções aplicadas (ver aba Itens e CONFERENCIA-TEXTOS.md).</t>
+          <t>02/10/2026: as 4 correções aplicadas; em 03/10/2026, mais 2 (D2-038 e D2b-051) na conferência dos 28 itens restantes (ver aba Itens e CONFERENCIA-TEXTOS.md).</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr"/>
@@ -3967,7 +4081,11 @@
           <t>Confirmar a nova composição para atualizar o normas-rag-corpus.md e o texto.</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr"/>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>02/10/2026: corpus de 14 documentos confirmado; normas-rag-corpus.md e texto atualizados.</t>
+        </is>
+      </c>
       <c r="F5" s="6" t="inlineStr"/>
     </row>
     <row r="6">

</xml_diff>